<commit_message>
Add news story about knowledge mapping technique
Links to Dartmouth News article on mapping student conceptual
knowledge from short multiple-choice quizzes.

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/news.xlsx
+++ b/data/news.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F15"/>
+  <dimension ref="A1:F16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -451,292 +451,277 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2025-08-01</t>
+          <t>2026-03-24</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Claudia Gonciulea joins the lab!</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr"/>
+          <t>New technique maps what students know using short quizzes</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>https://home.dartmouth.edu/news/2026/03/new-technique-maps-what-students-know-using-short-quizzes</t>
+        </is>
+      </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>We've managed to recruit superstar-scientist Claudia Gonciulea to our incoming PhD student cohort at Dartmouth!</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>[&lt;a href="https://context-lab.com/people.html"&gt;READ CLAUDIA'S BIO&lt;/a&gt;]</t>
+          <t>Dartmouth researchers have developed a mathematical technique for mapping a student's conceptual knowledge from their performance on short multiple-choice quizzes, creating a detailed topography that captures both areas of mastery and struggle.</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>claudia-gonciulea.png</t>
+          <t>map2.png</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2025-01-10</t>
+          <t>2025-08-01</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Why are we so preoccupied by the past?</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>https://www.scientificamerican.com/article/why-were-so-preoccupied-by-the-past/</t>
+          <t>Claudia Gonciulea joins the lab!</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Check out our reflection on our &lt;a href="https://www.nature.com/articles/s41467-024-52627-5" target="_blank"&gt;recent paper on prediction and retrodiction&lt;/a&gt; in &lt;a href="https://www.scientificamerican.com/article/why-were-so-preoccupied-by-the-past/" target="_blank"&gt;Scientific American&lt;/a&gt;!</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr"/>
+          <t>We've managed to recruit superstar-scientist Claudia Gonciulea to our incoming PhD student cohort at Dartmouth!</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>[&lt;a href="https://context-lab.com/people.html"&gt;READ CLAUDIA'S BIO&lt;/a&gt;]</t>
+        </is>
+      </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>scientific-american-past.png</t>
+          <t>claudia-gonciulea.png</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2024-07-01</t>
+          <t>2025-01-10</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Jeremy gets tenure!</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr"/>
+          <t>Why are we so preoccupied by the past?</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>https://www.scientificamerican.com/article/why-were-so-preoccupied-by-the-past/</t>
+        </is>
+      </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Jeremy managed to &lt;a href="https://home.dartmouth.edu/news/2024/08/more-60-professors-promoted-across-dartmouth" target="_blank"&gt;sneak past the tenure review committee&lt;/a&gt;-- they never even noticed he was actually three kittens in a lab coat! He even picked up some &lt;a href="https://home.dartmouth.edu/news/2024/07/celebrating-excellence-2024-faculty-awards" target="_blank"&gt;awards&lt;/a&gt; along the way.</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr"/>
+          <t>Check out our reflection on our &lt;a href="https://www.nature.com/articles/s41467-024-52627-5" target="_blank"&gt;recent paper on prediction and retrodiction&lt;/a&gt; in &lt;a href="https://www.scientificamerican.com/article/why-were-so-preoccupied-by-the-past/" target="_blank"&gt;Scientific American&lt;/a&gt;!</t>
+        </is>
+      </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>jeremy-tenure.png</t>
+          <t>scientific-american-past.png</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2022-01-25</t>
+          <t>2024-07-01</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>We CAREER'd!</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr"/>
+          <t>Jeremy gets tenure!</t>
+        </is>
+      </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>The CDL was awarded an &lt;a href="https://www.nsf.gov/awardsearch/show-award/?AWD_ID=2145172&amp;HistoricalAwards=false" target="_blank"&gt;NSF CAREER Award&lt;/a&gt; to map and enhance how students learn, using natural language processing models. We're excited to do some awesome science with our new-found riches!</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr"/>
+          <t>Jeremy managed to &lt;a href="https://home.dartmouth.edu/news/2024/08/more-60-professors-promoted-across-dartmouth" target="_blank"&gt;sneak past the tenure review committee&lt;/a&gt;-- they never even noticed he was actually three kittens in a lab coat! He even picked up some &lt;a href="https://home.dartmouth.edu/news/2024/07/celebrating-excellence-2024-faculty-awards" target="_blank"&gt;awards&lt;/a&gt; along the way.</t>
+        </is>
+      </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>nsf-career.png</t>
+          <t>jeremy-tenure.png</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2021-04-15</t>
+          <t>2022-01-25</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Paxton Fitzpatrick and Xinming Xu transform into graduate students</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>people.html</t>
+          <t>We CAREER'd!</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>We are excited to announce that Paxton Fitzpatrick (current role: lab manager) and Xinming Xu (current role: research assistant) will continue on in the Contextual Dynamics Lab as part of the 2021 graduate student class at Dartmouth!</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>[&lt;a href="people.html"&gt;READ PAXTON'S AND XINMING'S BIOS&lt;/a&gt;]</t>
+          <t>The CDL was awarded an &lt;a href="https://www.nsf.gov/awardsearch/show-award/?AWD_ID=2145172&amp;HistoricalAwards=false" target="_blank"&gt;NSF CAREER Award&lt;/a&gt; to map and enhance how students learn, using natural language processing models. We're excited to do some awesome science with our new-found riches!</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>paxton-xinming-grad.gif</t>
+          <t>nsf-career.png</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2021-03-01</t>
+          <t>2021-04-15</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>How do our memories take shape?</t>
+          <t>Paxton Fitzpatrick and Xinming Xu transform into graduate students</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>https://socialsciences.nature.com/posts/how-is-experience-transformed-into-memory</t>
+          <t>people.html</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>We've written a short piece on our &lt;a href="https://www.nature.com/articles/s41562-021-01051-6" target="_blank"&gt;&lt;em&gt;Sherlock&lt;/em&gt; paper&lt;/a&gt;— check it out &lt;a href="https://socialsciences.nature.com/posts/how-is-experience-transformed-into-memory" target="_blank"&gt;here&lt;/a&gt; on the &lt;a href="https://socialsciences.nature.com/" target="_blank"&gt;Nature Research Behavioural &amp; Social Sciences blog&lt;/a&gt;!</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr"/>
+          <t>We are excited to announce that Paxton Fitzpatrick (current role: lab manager) and Xinming Xu (current role: research assistant) will continue on in the Contextual Dynamics Lab as part of the 2021 graduate student class at Dartmouth!</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>[&lt;a href="people.html"&gt;READ PAXTON'S AND XINMING'S BIOS&lt;/a&gt;]</t>
+        </is>
+      </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>sherlock-memories.png</t>
+          <t>paxton-xinming-grad.gif</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2021-01-15</t>
+          <t>2021-03-01</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>CDL Undergraduate Researcher Will Baxley is Named a Goldwater Scholar</t>
+          <t>How do our memories take shape?</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>http://dartgo.org/dnewstwogoldwaters4</t>
+          <t>https://socialsciences.nature.com/posts/how-is-experience-transformed-into-memory</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Will Baxley was one of 396 undergraduates from around the country to receive a Goldwater Scholarship. The award "seeks to identify and support college sophomores and juniors who show exceptional promise of becoming this nation's next generation of research leaders" in the natural sciences, engineering, and mathematics. Go Will— we're proud of you!</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>[&lt;a href="people.html"&gt;READ WILL'S BIO&lt;/a&gt;]</t>
+          <t>We've written a short piece on our &lt;a href="https://www.nature.com/articles/s41562-021-01051-6" target="_blank"&gt;&lt;em&gt;Sherlock&lt;/em&gt; paper&lt;/a&gt;— check it out &lt;a href="https://socialsciences.nature.com/posts/how-is-experience-transformed-into-memory" target="_blank"&gt;here&lt;/a&gt; on the &lt;a href="https://socialsciences.nature.com/" target="_blank"&gt;Nature Research Behavioural &amp; Social Sciences blog&lt;/a&gt;!</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>will-baxley-goldwater.png</t>
+          <t>sherlock-memories.png</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2019-10-25</t>
+          <t>2021-01-15</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>We came, we saw, we Sfn'd</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr"/>
+          <t>CDL Undergraduate Researcher Will Baxley is Named a Goldwater Scholar</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>http://dartgo.org/dnewstwogoldwaters4</t>
+        </is>
+      </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>The CDL helped educate the neuroscience-enthusiast masses by presenting four posters at this year's SfN annual meeting. We also helped support the local economy by sampling some of Chicago's dining establishments. Go us!</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr"/>
+          <t>Will Baxley was one of 396 undergraduates from around the country to receive a Goldwater Scholarship. The award "seeks to identify and support college sophomores and juniors who show exceptional promise of becoming this nation's next generation of research leaders" in the natural sciences, engineering, and mathematics. Go Will— we're proud of you!</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>[&lt;a href="people.html"&gt;READ WILL'S BIO&lt;/a&gt;]</t>
+        </is>
+      </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>sfn-2019.png</t>
+          <t>will-baxley-goldwater.png</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2019-09-15</t>
+          <t>2019-10-25</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Timecorr toolbox unleashed upon an unsuspecting populace</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>http://timecorr.readthedocs.io/en/latest/</t>
+          <t>We came, we saw, we Sfn'd</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>We are thrilled to announce our new Python "Timecorr" toolbox for inferring dynamic high-order correlations in multivariate timeseries data. Check out the toolbox &lt;a href="http://timecorr.readthedocs.io/en/latest/" target="_blank"&gt;here&lt;/a&gt;, or our preprint &lt;a href="https://www.biorxiv.org/content/10.1101/763821v1" target="_blank"&gt;here&lt;/a&gt;!</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr"/>
+          <t>The CDL helped educate the neuroscience-enthusiast masses by presenting four posters at this year's SfN annual meeting. We also helped support the local economy by sampling some of Chicago's dining establishments. Go us!</t>
+        </is>
+      </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>timecorr.gif</t>
+          <t>sfn-2019.png</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2019-08-01</t>
+          <t>2019-09-15</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>CDL welcomes grad student Caroline Lee</t>
+          <t>Timecorr toolbox unleashed upon an unsuspecting populace</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>people.html</t>
+          <t>http://timecorr.readthedocs.io/en/latest/</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>We are excited to welcome Caroline Lee to the Contextual Dynamics Lab and the 2019 graduate student class at Dartmouth!</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>[&lt;a href="people.html"&gt;READ CAROLINE'S BIO&lt;/a&gt;]</t>
+          <t>We are thrilled to announce our new Python "Timecorr" toolbox for inferring dynamic high-order correlations in multivariate timeseries data. Check out the toolbox &lt;a href="http://timecorr.readthedocs.io/en/latest/" target="_blank"&gt;here&lt;/a&gt;, or our preprint &lt;a href="https://www.biorxiv.org/content/10.1101/763821v1" target="_blank"&gt;here&lt;/a&gt;!</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>caroline-lee.png</t>
+          <t>timecorr.gif</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2019-06-01</t>
+          <t>2019-08-01</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>The CDL snagged a new lab manager!</t>
+          <t>CDL welcomes grad student Caroline Lee</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -746,95 +731,123 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>We are excited to announce our awesome new lab manager: Paxton Fitzpatrick! Paxton is an old hand in the lab, having risen up through our ranks as an undergraduate research assistant. We are thrilled that he has decided to stay on in the lab and continue helping us to achieve our best science!</t>
+          <t>We are excited to welcome Caroline Lee to the Contextual Dynamics Lab and the 2019 graduate student class at Dartmouth!</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>[&lt;a href="people.html"&gt;READ PAXTON'S BIO&lt;/a&gt;]</t>
+          <t>[&lt;a href="people.html"&gt;READ CAROLINE'S BIO&lt;/a&gt;]</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>paxton-lab-manager.png</t>
+          <t>caroline-lee.png</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2019-03-01</t>
+          <t>2019-06-01</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>We want YOU to help manage our lab!</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr"/>
+          <t>The CDL snagged a new lab manager!</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>people.html</t>
+        </is>
+      </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>We're looking for a new lab manager! Read on for details...</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr"/>
+          <t>We are excited to announce our awesome new lab manager: Paxton Fitzpatrick! Paxton is an old hand in the lab, having risen up through our ranks as an undergraduate research assistant. We are thrilled that he has decided to stay on in the lab and continue helping us to achieve our best science!</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>[&lt;a href="people.html"&gt;READ PAXTON'S BIO&lt;/a&gt;]</t>
+        </is>
+      </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>lab-manager-wanted.jpg</t>
+          <t>paxton-lab-manager.png</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2018-05-15</t>
+          <t>2019-03-01</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>HyperTools in the news!</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>https://www.eurekalert.org/pub_releases/2018-05/dc-nsh050718.php</t>
+          <t>We want YOU to help manage our lab!</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Our HyperTools Python package for gaining geometric insights into high dimensional data is in the news! Press release &lt;a href="https://www.eurekalert.org/pub_releases/2018-05/dc-nsh050718.php" target="_blank"&gt;here&lt;/a&gt;; download &lt;a href="http://hypertools.readthedocs.io/" target="_blank"&gt;here&lt;/a&gt;.</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr"/>
+          <t>We're looking for a new lab manager! Read on for details...</t>
+        </is>
+      </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>hypertools.gif</t>
+          <t>lab-manager-wanted.jpg</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
+          <t>2018-05-15</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>HyperTools in the news!</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>https://www.eurekalert.org/pub_releases/2018-05/dc-nsh050718.php</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Our HyperTools Python package for gaining geometric insights into high dimensional data is in the news! Press release &lt;a href="https://www.eurekalert.org/pub_releases/2018-05/dc-nsh050718.php" target="_blank"&gt;here&lt;/a&gt;; download &lt;a href="http://hypertools.readthedocs.io/" target="_blank"&gt;here&lt;/a&gt;.</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>hypertools.gif</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
           <t>2018-03-01</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
+      <c r="B16" t="inlineStr">
         <is>
           <t>SuperEEG toolbox released!</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr">
+      <c r="C16" t="inlineStr">
         <is>
           <t>http://supereeg.readthedocs.io/en/latest/</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr">
+      <c r="D16" t="inlineStr">
         <is>
           <t>We are excited to announce our new Python "SuperEEG" toolbox for inferring whole-brain activity from a small(ish) number of ECoG electrodes. Check it out &lt;a href="http://supereeg.readthedocs.io/en/latest/" target="_blank"&gt;here&lt;/a&gt;!</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr"/>
-      <c r="F15" t="inlineStr">
+      <c r="F16" t="inlineStr">
         <is>
           <t>supereeg.gif</t>
         </is>

</xml_diff>

<commit_message>
Add the NSF museum-labels grant to the CV and lab news
NSF award 2604009, "AI Generated Interpretive Labels for Exhibits to
support engagement and learning in science museums" -- $900,000, PI,
with Joyce Ma (Exploratorium) as co-PI, running 2026-08-15 through
2029-07-31. Details came from the NSF award API rather than the award
page, which is a JS app that serves an empty shell to fetchers.

The news thumbnail is center-cropped to square on the museum and
resized to 300x300, with every other frame dropped (65 frames at 100ms,
same apparent speed) to bring it from 8.0MB down to 2.1MB. gifsicle's
--lossy speckled the flat cartoon colors, so this one is lossless.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RA2V7NZ1hQ4fQSoZcBQgHp
</commit_message>
<xml_diff>
--- a/data/news.xlsx
+++ b/data/news.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F16"/>
+  <dimension ref="A1:F17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -451,309 +451,309 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-03-24</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>New technique maps what students know using short quizzes</t>
+          <t>CDL and Exploratorium join forces to make science museums more awesome!</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>https://home.dartmouth.edu/news/2026/03/new-technique-maps-what-students-know-using-short-quizzes</t>
+          <t>https://www.nsf.gov/awardsearch/show-award/?AWD_ID=2604009</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Dartmouth researchers have developed a mathematical technique for mapping a student's conceptual knowledge from their performance on short multiple-choice quizzes, creating a detailed topography that captures both areas of mastery and struggle.</t>
+          <t>We're teaming up with the &lt;a href="https://www.exploratorium.edu/" target="_blank"&gt;Exploratorium&lt;/a&gt; on our next big project: museum exhibits that adapt on-the-fly to each visitor's unique interests, goals and background knowledge. We'll build &lt;a href="https://context-lab.com/mapper/" target="_blank"&gt;knowledge maps&lt;/a&gt; for each visitor and use them to customize what text they see at exhibits. We are grateful to the NSF for &lt;a href="https://www.nsf.gov/awardsearch/show-award/?AWD_ID=2604009" target="_blank"&gt;funding this project&lt;/a&gt;!</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>[&lt;a href="https://www.nsf.gov/awardsearch/show-award/?AWD_ID=2604009" target="_blank"&gt;READ THE ABSTRACT&lt;/a&gt;]</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>map2.png</t>
+          <t>nsf-museum-labels.gif</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2025-08-01</t>
+          <t>2026-03-24</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Claudia Gonciulea joins the lab!</t>
+          <t>New technique maps what students know using short quizzes</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>https://home.dartmouth.edu/news/2026/03/new-technique-maps-what-students-know-using-short-quizzes</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>We've managed to recruit superstar-scientist Claudia Gonciulea to our incoming PhD student cohort at Dartmouth!</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>[&lt;a href="https://context-lab.com/people.html"&gt;READ CLAUDIA'S BIO&lt;/a&gt;]</t>
+          <t>Dartmouth researchers have developed a mathematical technique for mapping a student's conceptual knowledge from their performance on short multiple-choice quizzes, creating a detailed topography that captures both areas of mastery and struggle.</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>claudia-gonciulea.png</t>
+          <t>map2.png</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2025-01-10</t>
+          <t>2025-08-01</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Why are we so preoccupied by the past?</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>https://www.scientificamerican.com/article/why-were-so-preoccupied-by-the-past/</t>
+          <t>Claudia Gonciulea joins the lab!</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Check out our reflection on our &lt;a href="https://www.nature.com/articles/s41467-024-52627-5" target="_blank"&gt;recent paper on prediction and retrodiction&lt;/a&gt; in &lt;a href="https://www.scientificamerican.com/article/why-were-so-preoccupied-by-the-past/" target="_blank"&gt;Scientific American&lt;/a&gt;!</t>
+          <t>We've managed to recruit superstar-scientist Claudia Gonciulea to our incoming PhD student cohort at Dartmouth!</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>[&lt;a href="https://context-lab.com/people.html"&gt;READ CLAUDIA'S BIO&lt;/a&gt;]</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>scientific-american-past.png</t>
+          <t>claudia-gonciulea.png</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2024-07-01</t>
+          <t>2025-01-10</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Jeremy gets tenure!</t>
+          <t>Why are we so preoccupied by the past?</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>https://www.scientificamerican.com/article/why-were-so-preoccupied-by-the-past/</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Jeremy managed to &lt;a href="https://home.dartmouth.edu/news/2024/08/more-60-professors-promoted-across-dartmouth" target="_blank"&gt;sneak past the tenure review committee&lt;/a&gt;-- they never even noticed he was actually three kittens in a lab coat! He even picked up some &lt;a href="https://home.dartmouth.edu/news/2024/07/celebrating-excellence-2024-faculty-awards" target="_blank"&gt;awards&lt;/a&gt; along the way.</t>
+          <t>Check out our reflection on our &lt;a href="https://www.nature.com/articles/s41467-024-52627-5" target="_blank"&gt;recent paper on prediction and retrodiction&lt;/a&gt; in &lt;a href="https://www.scientificamerican.com/article/why-were-so-preoccupied-by-the-past/" target="_blank"&gt;Scientific American&lt;/a&gt;!</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>jeremy-tenure.png</t>
+          <t>scientific-american-past.png</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2022-01-25</t>
+          <t>2024-07-01</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>We CAREER'd!</t>
+          <t>Jeremy gets tenure!</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>The CDL was awarded an &lt;a href="https://www.nsf.gov/awardsearch/show-award/?AWD_ID=2145172&amp;HistoricalAwards=false" target="_blank"&gt;NSF CAREER Award&lt;/a&gt; to map and enhance how students learn, using natural language processing models. We're excited to do some awesome science with our new-found riches!</t>
+          <t>Jeremy managed to &lt;a href="https://home.dartmouth.edu/news/2024/08/more-60-professors-promoted-across-dartmouth" target="_blank"&gt;sneak past the tenure review committee&lt;/a&gt;-- they never even noticed he was actually three kittens in a lab coat! He even picked up some &lt;a href="https://home.dartmouth.edu/news/2024/07/celebrating-excellence-2024-faculty-awards" target="_blank"&gt;awards&lt;/a&gt; along the way.</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>nsf-career.png</t>
+          <t>jeremy-tenure.png</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2021-04-15</t>
+          <t>2022-01-25</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Paxton Fitzpatrick and Xinming Xu transform into graduate students</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>people.html</t>
+          <t>We CAREER'd!</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>We are excited to announce that Paxton Fitzpatrick (current role: lab manager) and Xinming Xu (current role: research assistant) will continue on in the Contextual Dynamics Lab as part of the 2021 graduate student class at Dartmouth!</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>[&lt;a href="people.html"&gt;READ PAXTON'S AND XINMING'S BIOS&lt;/a&gt;]</t>
+          <t>The CDL was awarded an &lt;a href="https://www.nsf.gov/awardsearch/show-award/?AWD_ID=2145172&amp;HistoricalAwards=false" target="_blank"&gt;NSF CAREER Award&lt;/a&gt; to map and enhance how students learn, using natural language processing models. We're excited to do some awesome science with our new-found riches!</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>paxton-xinming-grad.gif</t>
+          <t>nsf-career.png</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2021-03-01</t>
+          <t>2021-04-15</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>How do our memories take shape?</t>
+          <t>Paxton Fitzpatrick and Xinming Xu transform into graduate students</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>https://socialsciences.nature.com/posts/how-is-experience-transformed-into-memory</t>
+          <t>people.html</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>We've written a short piece on our &lt;a href="https://www.nature.com/articles/s41562-021-01051-6" target="_blank"&gt;&lt;em&gt;Sherlock&lt;/em&gt; paper&lt;/a&gt;— check it out &lt;a href="https://socialsciences.nature.com/posts/how-is-experience-transformed-into-memory" target="_blank"&gt;here&lt;/a&gt; on the &lt;a href="https://socialsciences.nature.com/" target="_blank"&gt;Nature Research Behavioural &amp; Social Sciences blog&lt;/a&gt;!</t>
+          <t>We are excited to announce that Paxton Fitzpatrick (current role: lab manager) and Xinming Xu (current role: research assistant) will continue on in the Contextual Dynamics Lab as part of the 2021 graduate student class at Dartmouth!</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>[&lt;a href="people.html"&gt;READ PAXTON'S AND XINMING'S BIOS&lt;/a&gt;]</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>sherlock-memories.png</t>
+          <t>paxton-xinming-grad.gif</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2021-01-15</t>
+          <t>2021-03-01</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>CDL Undergraduate Researcher Will Baxley is Named a Goldwater Scholar</t>
+          <t>How do our memories take shape?</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>http://dartgo.org/dnewstwogoldwaters4</t>
+          <t>https://socialsciences.nature.com/posts/how-is-experience-transformed-into-memory</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Will Baxley was one of 396 undergraduates from around the country to receive a Goldwater Scholarship. The award "seeks to identify and support college sophomores and juniors who show exceptional promise of becoming this nation's next generation of research leaders" in the natural sciences, engineering, and mathematics. Go Will— we're proud of you!</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>[&lt;a href="people.html"&gt;READ WILL'S BIO&lt;/a&gt;]</t>
+          <t>We've written a short piece on our &lt;a href="https://www.nature.com/articles/s41562-021-01051-6" target="_blank"&gt;&lt;em&gt;Sherlock&lt;/em&gt; paper&lt;/a&gt;— check it out &lt;a href="https://socialsciences.nature.com/posts/how-is-experience-transformed-into-memory" target="_blank"&gt;here&lt;/a&gt; on the &lt;a href="https://socialsciences.nature.com/" target="_blank"&gt;Nature Research Behavioural &amp; Social Sciences blog&lt;/a&gt;!</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>will-baxley-goldwater.png</t>
+          <t>sherlock-memories.png</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2019-10-25</t>
+          <t>2021-01-15</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>We came, we saw, we Sfn'd</t>
+          <t>CDL Undergraduate Researcher Will Baxley is Named a Goldwater Scholar</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>http://dartgo.org/dnewstwogoldwaters4</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>The CDL helped educate the neuroscience-enthusiast masses by presenting four posters at this year's SfN annual meeting. We also helped support the local economy by sampling some of Chicago's dining establishments. Go us!</t>
+          <t>Will Baxley was one of 396 undergraduates from around the country to receive a Goldwater Scholarship. The award "seeks to identify and support college sophomores and juniors who show exceptional promise of becoming this nation's next generation of research leaders" in the natural sciences, engineering, and mathematics. Go Will— we're proud of you!</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>[&lt;a href="people.html"&gt;READ WILL'S BIO&lt;/a&gt;]</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>sfn-2019.png</t>
+          <t>will-baxley-goldwater.png</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2019-09-15</t>
+          <t>2019-10-25</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Timecorr toolbox unleashed upon an unsuspecting populace</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>http://timecorr.readthedocs.io/en/latest/</t>
+          <t>We came, we saw, we Sfn'd</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>We are thrilled to announce our new Python "Timecorr" toolbox for inferring dynamic high-order correlations in multivariate timeseries data. Check out the toolbox &lt;a href="http://timecorr.readthedocs.io/en/latest/" target="_blank"&gt;here&lt;/a&gt;, or our preprint &lt;a href="https://www.biorxiv.org/content/10.1101/763821v1" target="_blank"&gt;here&lt;/a&gt;!</t>
+          <t>The CDL helped educate the neuroscience-enthusiast masses by presenting four posters at this year's SfN annual meeting. We also helped support the local economy by sampling some of Chicago's dining establishments. Go us!</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>timecorr.gif</t>
+          <t>sfn-2019.png</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2019-08-01</t>
+          <t>2019-09-15</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>CDL welcomes grad student Caroline Lee</t>
+          <t>Timecorr toolbox unleashed upon an unsuspecting populace</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>people.html</t>
+          <t>http://timecorr.readthedocs.io/en/latest/</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>We are excited to welcome Caroline Lee to the Contextual Dynamics Lab and the 2019 graduate student class at Dartmouth!</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>[&lt;a href="people.html"&gt;READ CAROLINE'S BIO&lt;/a&gt;]</t>
+          <t>We are thrilled to announce our new Python "Timecorr" toolbox for inferring dynamic high-order correlations in multivariate timeseries data. Check out the toolbox &lt;a href="http://timecorr.readthedocs.io/en/latest/" target="_blank"&gt;here&lt;/a&gt;, or our preprint &lt;a href="https://www.biorxiv.org/content/10.1101/763821v1" target="_blank"&gt;here&lt;/a&gt;!</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>caroline-lee.png</t>
+          <t>timecorr.gif</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2019-06-01</t>
+          <t>2019-08-01</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>The CDL snagged a new lab manager!</t>
+          <t>CDL welcomes grad student Caroline Lee</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -763,91 +763,123 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>We are excited to announce our awesome new lab manager: Paxton Fitzpatrick! Paxton is an old hand in the lab, having risen up through our ranks as an undergraduate research assistant. We are thrilled that he has decided to stay on in the lab and continue helping us to achieve our best science!</t>
+          <t>We are excited to welcome Caroline Lee to the Contextual Dynamics Lab and the 2019 graduate student class at Dartmouth!</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>[&lt;a href="people.html"&gt;READ PAXTON'S BIO&lt;/a&gt;]</t>
+          <t>[&lt;a href="people.html"&gt;READ CAROLINE'S BIO&lt;/a&gt;]</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>paxton-lab-manager.png</t>
+          <t>caroline-lee.png</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2019-03-01</t>
+          <t>2019-06-01</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>We want YOU to help manage our lab!</t>
+          <t>The CDL snagged a new lab manager!</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>people.html</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>We're looking for a new lab manager! Read on for details...</t>
+          <t>We are excited to announce our awesome new lab manager: Paxton Fitzpatrick! Paxton is an old hand in the lab, having risen up through our ranks as an undergraduate research assistant. We are thrilled that he has decided to stay on in the lab and continue helping us to achieve our best science!</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>[&lt;a href="people.html"&gt;READ PAXTON'S BIO&lt;/a&gt;]</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>lab-manager-wanted.jpg</t>
+          <t>paxton-lab-manager.png</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2018-05-15</t>
+          <t>2019-03-01</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>HyperTools in the news!</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>https://www.eurekalert.org/pub_releases/2018-05/dc-nsh050718.php</t>
+          <t>We want YOU to help manage our lab!</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Our HyperTools Python package for gaining geometric insights into high dimensional data is in the news! Press release &lt;a href="https://www.eurekalert.org/pub_releases/2018-05/dc-nsh050718.php" target="_blank"&gt;here&lt;/a&gt;; download &lt;a href="http://hypertools.readthedocs.io/" target="_blank"&gt;here&lt;/a&gt;.</t>
+          <t>We're looking for a new lab manager! Read on for details...</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>hypertools.gif</t>
+          <t>lab-manager-wanted.jpg</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
+          <t>2018-05-15</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>HyperTools in the news!</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>https://www.eurekalert.org/pub_releases/2018-05/dc-nsh050718.php</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Our HyperTools Python package for gaining geometric insights into high dimensional data is in the news! Press release &lt;a href="https://www.eurekalert.org/pub_releases/2018-05/dc-nsh050718.php" target="_blank"&gt;here&lt;/a&gt;; download &lt;a href="http://hypertools.readthedocs.io/" target="_blank"&gt;here&lt;/a&gt;.</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>hypertools.gif</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
           <t>2018-03-01</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr">
+      <c r="B17" t="inlineStr">
         <is>
           <t>SuperEEG toolbox released!</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr">
+      <c r="C17" t="inlineStr">
         <is>
           <t>http://supereeg.readthedocs.io/en/latest/</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr">
+      <c r="D17" t="inlineStr">
         <is>
           <t>We are excited to announce our new Python "SuperEEG" toolbox for inferring whole-brain activity from a small(ish) number of ECoG electrodes. Check it out &lt;a href="http://supereeg.readthedocs.io/en/latest/" target="_blank"&gt;here&lt;/a&gt;!</t>
         </is>
       </c>
-      <c r="F16" t="inlineStr">
+      <c r="F17" t="inlineStr">
         <is>
           <t>supereeg.gif</t>
         </is>

</xml_diff>